<commit_message>
refactor(pricing)!: align requests and Excel APIs
BREAKING CHANGE: request FairRate(index) and read the single fair_rate
result. Indices select swap legs or loan rate segments; evaluate each
target separately. Remove the ambiguous fair_rates result array.

Expose separate Excel instrument, trade, policy, pricer and result
objects. Select ordinary funding curves through native discount policies.
Keep loan contract terms and pricer settings in typed worksheet ranges.

Regenerate workbooks and update native, Python and Excel examples.
</commit_message>
<xml_diff>
--- a/bindings/excel/examples/bond_pricing_example.xlsx
+++ b/bindings/excel/examples/bond_pricing_example.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="44">
   <si>
     <t>Straight bonds: price anchors, duration, spread, and curve risk</t>
   </si>
@@ -55,7 +55,7 @@
     <t>Compare the same fixed bond anchored at zero Z-spread, 100 bp Z-spread, and clean price 100.</t>
   </si>
   <si>
-    <t>QS.BOND.PRICE is monetary PV; CleanPrice/DirtyPrice anchors use quotation units per 100 face.</t>
+    <t>QS.RESULT.VALUE is monetary PV; CleanPrice/DirtyPrice anchors use quotation units per 100 face.</t>
   </si>
   <si>
     <t>Duration is yield-modified duration. Spread derivatives and curve derivatives retain their actual units.</t>
@@ -127,6 +127,27 @@
     <t>Coupon</t>
   </si>
   <si>
+    <t>USD</t>
+  </si>
+  <si>
+    <t>SOFR</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>ModifiedDuration</t>
+  </si>
+  <si>
+    <t>ZSpread</t>
+  </si>
+  <si>
+    <t>Cashflows</t>
+  </si>
+  <si>
+    <t>Sensitivities</t>
+  </si>
+  <si>
     <t>Anchor</t>
   </si>
   <si>
@@ -145,7 +166,7 @@
     <t>Z-spread</t>
   </si>
   <si>
-    <t>ZSpread</t>
+    <t>Evaluation results</t>
   </si>
   <si>
     <t>CleanPrice</t>
@@ -636,7 +657,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A3:L14"/>
+  <dimension ref="A3:L24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="4" width="22.7109375" style="1" customWidth="1"/>
@@ -645,7 +666,7 @@
     <col min="7" max="12" width="22.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:9">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -660,7 +681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:9">
       <c r="E4" s="1" t="s">
         <v>13</v>
       </c>
@@ -669,7 +690,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:9">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -677,7 +698,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:9">
       <c r="A6" s="3" t="s">
         <v>18</v>
       </c>
@@ -692,7 +713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:9">
       <c r="A7" s="3" t="s">
         <v>19</v>
       </c>
@@ -700,7 +721,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:9">
       <c r="A8" s="3" t="s">
         <v>20</v>
       </c>
@@ -708,7 +729,7 @@
         <v>0.032</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:9">
       <c r="A9" s="3" t="s">
         <v>21</v>
       </c>
@@ -716,7 +737,7 @@
         <v>0.034</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:9">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -724,7 +745,7 @@
         <v>0.035</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:9">
       <c r="E11" s="1" t="s">
         <v>15</v>
       </c>
@@ -733,7 +754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:9">
       <c r="E12" s="1" t="s">
         <v>16</v>
       </c>
@@ -742,9 +763,52 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:9">
       <c r="A14" s="1" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="F15" cm="1">
+        <f t="array" ref="F15">_xll.QS.DISCOUNT.POLICY.FIXED.INCOME("Bonds.Policy",H15:I15)</f>
+        <v>0</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="F16" cm="1">
+        <f t="array" ref="F16">_xll.QS.PRICER.CREATE("Bonds.Pricer","BondPricer",F15)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="8:8">
+      <c r="H20" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" spans="8:8">
+      <c r="H21" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" spans="8:8">
+      <c r="H22" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="8:8">
+      <c r="H23" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24" spans="8:8">
+      <c r="H24" s="1" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -760,15 +824,19 @@
     <col min="1" max="12" width="22.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:4">
       <c r="A4" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" spans="1:2">
+      <c r="D4" s="1" cm="1">
+        <f t="array" ref="D4">_xll.QS.INSTRUMENT.FIXED.BOND("Bonds.Instrument",B4,B5,"USD","",B6,B7,"Actual360","Compounded","Semiannual","Semiannual")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5" s="1" t="s">
         <v>24</v>
       </c>
@@ -776,7 +844,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
         <v>26</v>
       </c>
@@ -784,7 +852,7 @@
         <v>1000000</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
         <v>27</v>
       </c>
@@ -807,95 +875,110 @@
     <col min="4" max="12" width="22.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:7">
       <c r="A4" s="5" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F4" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" s="3" t="s">
-        <v>34</v>
-      </c>
       <c r="B5" s="3">
         <v>0</v>
       </c>
       <c r="C5" cm="1">
-        <f t="array" ref="C5">_xll.QS.TRADE.FIXED.BOND("Bonds.Case5",Market!$B$3,'Bond Inputs'!$B$4,'Bond Inputs'!$B$5,"USD","SOFR",'Bond Inputs'!$B$6,'Bond Inputs'!$B$7,"Receive","Actual360","Compounded","Semiannual","Semiannual",A5,B5)</f>
+        <f t="array" ref="C5">_xll.QS.TRADE.CREATE("Bonds.Case5",'Bond Inputs'!$D$4,Market!$B$3,"Receive",,,A5,B5)</f>
         <v>0</v>
       </c>
       <c r="D5" s="6" cm="1">
-        <f t="array" ref="D5">_xll.QS.BOND.PRICE(C5,Market!$F$11)</f>
+        <f t="array" ref="D5">_xll.QS.RESULT.VALUE(G5)</f>
         <v>0</v>
       </c>
       <c r="E5" s="6" cm="1">
-        <f t="array" ref="E5">_xll.QS.BOND.MODIFIED.DURATION(C5,Market!$F$11)</f>
+        <f t="array" ref="E5">_xll.QS.RESULT.MODIFIED.DURATION(G5)</f>
         <v>0</v>
       </c>
       <c r="F5" s="7" cm="1">
-        <f t="array" ref="F5">_xll.QS.BOND.Z.SPREAD(C5,Market!$F$11)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+        <f t="array" ref="F5">_xll.QS.RESULT.Z.SPREAD(G5)</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="1" cm="1">
+        <f t="array" ref="G5">_xll.QS.EVALUATE("Bonds.Results5",Market!$F$16,C5,Market!$F$11,Market!$H$20:$H$24)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
       <c r="A6" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B6" s="3">
         <v>0.01</v>
       </c>
       <c r="C6" cm="1">
-        <f t="array" ref="C6">_xll.QS.TRADE.FIXED.BOND("Bonds.Case6",Market!$B$3,'Bond Inputs'!$B$4,'Bond Inputs'!$B$5,"USD","SOFR",'Bond Inputs'!$B$6,'Bond Inputs'!$B$7,"Receive","Actual360","Compounded","Semiannual","Semiannual",A6,B6)</f>
+        <f t="array" ref="C6">_xll.QS.TRADE.CREATE("Bonds.Case6",'Bond Inputs'!$D$4,Market!$B$3,"Receive",,,A6,B6)</f>
         <v>0</v>
       </c>
       <c r="D6" s="6" cm="1">
-        <f t="array" ref="D6">_xll.QS.BOND.PRICE(C6,Market!$F$11)</f>
+        <f t="array" ref="D6">_xll.QS.RESULT.VALUE(G6)</f>
         <v>0</v>
       </c>
       <c r="E6" s="6" cm="1">
-        <f t="array" ref="E6">_xll.QS.BOND.MODIFIED.DURATION(C6,Market!$F$11)</f>
+        <f t="array" ref="E6">_xll.QS.RESULT.MODIFIED.DURATION(G6)</f>
         <v>0</v>
       </c>
       <c r="F6" s="7" cm="1">
-        <f t="array" ref="F6">_xll.QS.BOND.Z.SPREAD(C6,Market!$F$11)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
+        <f t="array" ref="F6">_xll.QS.RESULT.Z.SPREAD(G6)</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="1" cm="1">
+        <f t="array" ref="G6">_xll.QS.EVALUATE("Bonds.Results6",Market!$F$16,C6,Market!$F$11,Market!$H$20:$H$24)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
       <c r="A7" s="3" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="B7" s="3">
         <v>100</v>
       </c>
       <c r="C7" cm="1">
-        <f t="array" ref="C7">_xll.QS.TRADE.FIXED.BOND("Bonds.Case7",Market!$B$3,'Bond Inputs'!$B$4,'Bond Inputs'!$B$5,"USD","SOFR",'Bond Inputs'!$B$6,'Bond Inputs'!$B$7,"Receive","Actual360","Compounded","Semiannual","Semiannual",A7,B7)</f>
+        <f t="array" ref="C7">_xll.QS.TRADE.CREATE("Bonds.Case7",'Bond Inputs'!$D$4,Market!$B$3,"Receive",,,A7,B7)</f>
         <v>0</v>
       </c>
       <c r="D7" s="6" cm="1">
-        <f t="array" ref="D7">_xll.QS.BOND.PRICE(C7,Market!$F$11)</f>
+        <f t="array" ref="D7">_xll.QS.RESULT.VALUE(G7)</f>
         <v>0</v>
       </c>
       <c r="E7" s="6" cm="1">
-        <f t="array" ref="E7">_xll.QS.BOND.MODIFIED.DURATION(C7,Market!$F$11)</f>
+        <f t="array" ref="E7">_xll.QS.RESULT.MODIFIED.DURATION(G7)</f>
         <v>0</v>
       </c>
       <c r="F7" s="7" cm="1">
-        <f t="array" ref="F7">_xll.QS.BOND.Z.SPREAD(C7,Market!$F$11)</f>
+        <f t="array" ref="F7">_xll.QS.RESULT.Z.SPREAD(G7)</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="1" cm="1">
+        <f t="array" ref="G7">_xll.QS.EVALUATE("Bonds.Results7",Market!$F$16,C7,Market!$F$11,Market!$H$20:$H$24)</f>
         <v>0</v>
       </c>
     </row>
@@ -914,7 +997,7 @@
   <sheetData>
     <row r="4" spans="1:1">
       <c r="A4" s="1" cm="1">
-        <f t="array" ref="A4">_xll.QS.CASHFLOWS(Valuation!C5,Market!F11)</f>
+        <f t="array" ref="A4">_xll.QS.RESULT.CASHFLOWS(Valuation!G5)</f>
         <v>0</v>
       </c>
     </row>
@@ -933,16 +1016,16 @@
   <sheetData>
     <row r="2" spans="1:5">
       <c r="E2" s="8" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" cm="1">
-        <f t="array" ref="A4">_xll.QS.BOND.SENSITIVITIES(Valuation!C6,Market!F11)</f>
+        <f t="array" ref="A4">_xll.QS.RESULT.SENSITIVITIES(Valuation!G6)</f>
         <v>0</v>
       </c>
       <c r="E4" s="1" cm="1">
-        <f t="array" ref="E4">_xll.QS.BOND.SENSITIVITIES(Valuation!C6,Market!F11,TRUE,FALSE)</f>
+        <f t="array" ref="E4">_xll.QS.RESULT.SENSITIVITIES(Valuation!G6,TRUE,FALSE)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(excel): manage workbook object lifetimes
Track cell contributions and dependencies, rebuild saved handles on open, and release closed workbook registries.

Add nonvolatile caching, direct policy arguments and scalar/batch PV APIs.
</commit_message>
<xml_diff>
--- a/bindings/excel/examples/bond_pricing_example.xlsx
+++ b/bindings/excel/examples/bond_pricing_example.xlsx
@@ -42,6 +42,8 @@
     <definedName name="Bond_Context">'3 Build'!$B$7</definedName>
     <definedName name="Bond_Coupon">'1 Inputs'!$B$11</definedName>
     <definedName name="Bond_Curves">Bond_BaseCurves</definedName>
+    <definedName name="Bond_DiscountCurrency">'1 Inputs'!$A$31</definedName>
+    <definedName name="Bond_DiscountIndex">'1 Inputs'!$B$31</definedName>
     <definedName name="Bond_DiscountMapping">'1 Inputs'!$A$31:$B$31</definedName>
     <definedName name="Bond_InitialCurves">'2 Market'!$B$21</definedName>
     <definedName name="Bond_InitialQuotes">'2 Market'!$B$18</definedName>
@@ -2194,7 +2196,7 @@
         <v>107</v>
       </c>
       <c r="B13" s="10" cm="1" t="str">
-        <f t="array" ref="B13">_xll.QS.DISCOUNT.POLICY.FIXED.INCOME("Bond.Policy",Bond_DiscountMapping)</f>
+        <f t="array" ref="B13">_xll.QS.DISCOUNT.POLICY.FIXED.INCOME("Bond.Policy",Bond_DiscountCurrency,Bond_DiscountIndex)</f>
         <v/>
       </c>
       <c r="C13" s="7" t="s">
@@ -2204,7 +2206,7 @@
     <row r="14" spans="1:3" ht="34" customHeight="1">
       <c r="A14" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B13),",",", ")</f>
-        <v>=QS.DISCOUNT.POLICY.FIXED.INCOME("Bond.Policy", Bond_DiscountMapping)</v>
+        <v>=QS.DISCOUNT.POLICY.FIXED.INCOME("Bond.Policy", Bond_DiscountCurrency, Bond_DiscountIndex)</v>
       </c>
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>

</xml_diff>

<commit_message>
docs(excel): add context-first pricing study
</commit_message>
<xml_diff>
--- a/bindings/excel/examples/bond_pricing_example.xlsx
+++ b/bindings/excel/examples/bond_pricing_example.xlsx
@@ -2156,7 +2156,7 @@
         <v>103</v>
       </c>
       <c r="B7" s="10" cm="1" t="str">
-        <f t="array" ref="B7">_xll.QS.CONTEXT.CREATE("Bond.Context",Bond_Quotes,Bond_Curves,,,,,,,,,,"USD","SOFR","Mid")</f>
+        <f t="array" ref="B7">_xll.QS.CONTEXT.FROM.COMPONENTS("Bond.Context",Bond_Quotes,Bond_Curves,,,,,,,,,,"USD","SOFR","Mid")</f>
         <v/>
       </c>
       <c r="C7" s="7" t="s">
@@ -2166,7 +2166,7 @@
     <row r="8" spans="1:3" ht="34" customHeight="1">
       <c r="A8" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B7),",",", ")</f>
-        <v>=QS.CONTEXT.CREATE("Bond.Context", Bond_Quotes, Bond_Curves, , , , , , , , , , "USD", "SOFR", "Mid")</v>
+        <v>=QS.CONTEXT.FROM.COMPONENTS("Bond.Context", Bond_Quotes, Bond_Curves, , , , , , , , , , "USD", "SOFR", "Mid")</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>

</xml_diff>

<commit_message>
docs(excel): migrate guides and workbooks
</commit_message>
<xml_diff>
--- a/bindings/excel/examples/bond_pricing_example.xlsx
+++ b/bindings/excel/examples/bond_pricing_example.xlsx
@@ -16,7 +16,7 @@
     <sheet name="6 Risk" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="Bond_BaseCurves">'2 Market'!$B$24</definedName>
+    <definedName name="Bond_BaseCurves">'2 Market'!$B$21</definedName>
     <definedName name="Bond_C01_Anchor">'1 Inputs'!$B$17</definedName>
     <definedName name="Bond_C01_AnchorValue">'1 Inputs'!$C$17</definedName>
     <definedName name="Bond_C01_Duration">'4 Results'!$C$7</definedName>
@@ -41,21 +41,19 @@
     <definedName name="Bond_CaseNames">'4 Results'!$A$7:$A$9</definedName>
     <definedName name="Bond_Context">'3 Build'!$B$7</definedName>
     <definedName name="Bond_Coupon">'1 Inputs'!$B$11</definedName>
-    <definedName name="Bond_Curves">Bond_BaseCurves</definedName>
     <definedName name="Bond_DiscountCurrency">'1 Inputs'!$A$31</definedName>
     <definedName name="Bond_DiscountIndex">'1 Inputs'!$B$31</definedName>
     <definedName name="Bond_DiscountMapping">'1 Inputs'!$A$31:$B$31</definedName>
-    <definedName name="Bond_InitialCurves">'2 Market'!$B$21</definedName>
-    <definedName name="Bond_InitialQuotes">'2 Market'!$B$18</definedName>
     <definedName name="Bond_Instrument">'3 Build'!$B$10</definedName>
+    <definedName name="Bond_MarketInputs">'2 Market'!$B$21:$B$23</definedName>
     <definedName name="Bond_Maturity">'1 Inputs'!$B$9</definedName>
     <definedName name="Bond_Notional">'1 Inputs'!$B$10</definedName>
     <definedName name="Bond_Pillars">'2 Market'!$A$7:$A$11</definedName>
     <definedName name="Bond_Policy">'3 Build'!$B$13</definedName>
     <definedName name="Bond_Pricer">'3 Build'!$B$16</definedName>
-    <definedName name="Bond_Quotes">Bond_InitialQuotes</definedName>
     <definedName name="Bond_Requests">'1 Inputs'!$A$23:$A$27</definedName>
     <definedName name="Bond_ResultHandles">'3 Build'!$B$40:$B$42</definedName>
+    <definedName name="Bond_Root">'2 Market'!$B$18</definedName>
     <definedName name="Bond_SelectedCase">'4 Results'!$B$13</definedName>
     <definedName name="Bond_SelectedResult">'3 Build'!$B$45</definedName>
     <definedName name="Bond_Side">'1 Inputs'!$B$12</definedName>
@@ -177,7 +175,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Sets the valuation date for the market.</t>
+          <t>Owns the market stores and date.</t>
         </r>
       </text>
     </comment>
@@ -190,20 +188,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Curve construction choices are separate from contract terms.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B24" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>The context builds this curve from the blue input range.</t>
+          <t>Every addition references the same root; fields are separate arrays.</t>
         </r>
       </text>
     </comment>
@@ -387,7 +372,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="142">
   <si>
     <t>Bond anchors · contract, trade and value</t>
   </si>
@@ -665,22 +650,16 @@
     <t>Why it is needed</t>
   </si>
   <si>
-    <t>1. Create quote store</t>
-  </si>
-  <si>
-    <t>Sets the valuation date for the market.</t>
-  </si>
-  <si>
-    <t>3. Create curve configurations</t>
-  </si>
-  <si>
-    <t>Curve construction choices are separate from contract terms.</t>
-  </si>
-  <si>
-    <t>4. Configure SOFR</t>
-  </si>
-  <si>
-    <t>The context builds this curve from the blue input range.</t>
+    <t>1. Create root context</t>
+  </si>
+  <si>
+    <t>Owns the market stores and date.</t>
+  </si>
+  <si>
+    <t>Add SOFR</t>
+  </si>
+  <si>
+    <t>Every addition references the same root; fields are separate arrays.</t>
   </si>
   <si>
     <t>Build one contract and three positions</t>
@@ -1911,7 +1890,7 @@
     <tabColor rgb="FF337AB7"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="24" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="38.7109375" style="1" customWidth="1"/>
@@ -2023,7 +2002,7 @@
         <v>92</v>
       </c>
       <c r="B18" s="10" cm="1" t="str">
-        <f t="array" ref="B18">_xll.QS.QUOTES.CREATE("Bond.Quotes",Bond_ValuationDate)</f>
+        <f t="array" ref="B18">_xll.QS.CONTEXT.CREATE("Bond.Root",Bond_ValuationDate,"USD","SOFR")</f>
         <v/>
       </c>
       <c r="C18" s="7" t="s">
@@ -2033,7 +2012,7 @@
     <row r="19" spans="1:3" ht="34" customHeight="1">
       <c r="A19" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B18),",",", ")</f>
-        <v>=QS.QUOTES.CREATE("Bond.Quotes", Bond_ValuationDate)</v>
+        <v>=QS.CONTEXT.CREATE("Bond.Root", Bond_ValuationDate, "USD", "SOFR")</v>
       </c>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
@@ -2043,7 +2022,7 @@
         <v>94</v>
       </c>
       <c r="B21" s="10" cm="1" t="str">
-        <f t="array" ref="B21">_xll.QS.CURVE.CONFIGS.CREATE("Bond.Curves")</f>
+        <f t="array" ref="B21">_xll.QS.CONTEXT.ADD.ZERO.CURVE(Bond_Root,"SOFR",Bond_Pillars,Bond_ZeroRates,"Actual360","Linear",TRUE,"Continuous","Annual")</f>
         <v/>
       </c>
       <c r="C21" s="7" t="s">
@@ -2053,39 +2032,18 @@
     <row r="22" spans="1:3" ht="34" customHeight="1">
       <c r="A22" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B21),",",", ")</f>
-        <v>=QS.CURVE.CONFIGS.CREATE("Bond.Curves")</v>
+        <v>=QS.CONTEXT.ADD.ZERO.CURVE(Bond_Root, "SOFR", Bond_Pillars, Bond_ZeroRates, "Actual360", "Linear", TRUE, "Continuous", "Annual")</v>
       </c>
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
     </row>
-    <row r="24" spans="1:3" ht="38" customHeight="1">
-      <c r="A24" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B24" s="10" cm="1" t="str">
-        <f t="array" ref="B24">_xll.QS.CURVE.CONFIGS.ADD.ZERO(Bond_InitialCurves,"SOFR","Actual360","Linear",TRUE,Bond_Pillars,Bond_ZeroRates,"Continuous","Annual")</f>
-        <v/>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="34" customHeight="1">
-      <c r="A25" s="13" t="str">
-        <f>SUBSTITUTE(_xlfn.FORMULATEXT(B24),",",", ")</f>
-        <v>=QS.CURVE.CONFIGS.ADD.ZERO(Bond_InitialCurves, "SOFR", "Actual360", "Linear", TRUE, Bond_Pillars, Bond_ZeroRates, "Continuous", "Annual")</v>
-      </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="5">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C3"/>
     <mergeCell ref="A13:C14"/>
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A22:C22"/>
-    <mergeCell ref="A25:C25"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" location="'Start Here'!A1" display="← Start Here"/>
@@ -2115,14 +2073,14 @@
   <sheetData>
     <row r="1" spans="1:3" ht="38" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="2" spans="1:3" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -2137,70 +2095,70 @@
         <v>36</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="36" customHeight="1">
       <c r="A6" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>90</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="38" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B7" s="10" cm="1" t="str">
-        <f t="array" ref="B7">_xll.QS.CONTEXT.FROM.COMPONENTS("Bond.Context",Bond_Quotes,Bond_Curves,,,,,,,,,,"USD","SOFR","Mid")</f>
+        <f t="array" ref="B7">_xll.QS.CONTEXT.PREPARE("Bond.Context",Bond_Root,Bond_MarketInputs)</f>
         <v/>
       </c>
       <c r="C7" s="7" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="34" customHeight="1">
       <c r="A8" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B7),",",", ")</f>
-        <v>=QS.CONTEXT.FROM.COMPONENTS("Bond.Context", Bond_Quotes, Bond_Curves, , , , , , , , , , "USD", "SOFR", "Mid")</v>
+        <v>=QS.CONTEXT.PREPARE("Bond.Context", Bond_Root, Bond_MarketInputs)</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
     </row>
     <row r="10" spans="1:3" ht="38" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B10" s="10" cm="1" t="str">
-        <f t="array" ref="B10">_xll.QS.INSTRUMENT.FIXED.BOND("Bond.Instrument",Bond_Start,Bond_Maturity,"USD",,Bond_Notional,Bond_Coupon,"Actual360","Compounded","Semiannual","Semiannual")</f>
+        <f t="array" ref="B10">_xll.QS.INSTRUMENT.FIXED.RATE.BOND("Bond.Instrument",Bond_Start,Bond_Maturity,"USD",,Bond_Notional,Bond_Coupon,"Actual360","Compounded","Semiannual","Semiannual")</f>
         <v/>
       </c>
       <c r="C10" s="7" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="34" customHeight="1">
       <c r="A11" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B10),",",", ")</f>
-        <v>=QS.INSTRUMENT.FIXED.BOND("Bond.Instrument", Bond_Start, Bond_Maturity, "USD", , Bond_Notional, Bond_Coupon, "Actual360", "Compounded", "Semiannual", "Semiannual")</v>
+        <v>=QS.INSTRUMENT.FIXED.RATE.BOND("Bond.Instrument", Bond_Start, Bond_Maturity, "USD", , Bond_Notional, Bond_Coupon, "Actual360", "Compounded", "Semiannual", "Semiannual")</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
     </row>
     <row r="13" spans="1:3" ht="38" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B13" s="10" cm="1" t="str">
         <f t="array" ref="B13">_xll.QS.DISCOUNT.POLICY.FIXED.INCOME("Bond.Policy",Bond_DiscountCurrency,Bond_DiscountIndex)</f>
         <v/>
       </c>
       <c r="C13" s="7" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="34" customHeight="1">
@@ -2213,14 +2171,14 @@
     </row>
     <row r="16" spans="1:3" ht="38" customHeight="1">
       <c r="A16" s="4" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B16" s="10" cm="1" t="str">
         <f t="array" ref="B16">_xll.QS.PRICER.CREATE("Bond.Pricer","BondPricer",Bond_Policy)</f>
         <v/>
       </c>
       <c r="C16" s="7" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="34" customHeight="1">
@@ -2233,14 +2191,14 @@
     </row>
     <row r="19" spans="1:3" ht="38" customHeight="1">
       <c r="A19" s="4" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B19" s="10" cm="1" t="str">
         <f t="array" ref="B19">_xll.QS.TRADE.CREATE("Bond.C01.Trade",Bond_Instrument,Bond_ValuationDate,Bond_Side,,,Bond_C01_Anchor,Bond_C01_AnchorValue)</f>
         <v/>
       </c>
       <c r="C19" s="7" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="34" customHeight="1">
@@ -2253,34 +2211,34 @@
     </row>
     <row r="22" spans="1:3" ht="38" customHeight="1">
       <c r="A22" s="4" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B22" s="10" cm="1" t="str">
-        <f t="array" ref="B22">_xll.QS.EVALUATE("Bond.C01.Result",Bond_Pricer,Bond_C01_Trade,Bond_Context,Bond_Requests)</f>
+        <f t="array" ref="B22">_xll.QS.EVALUATE.RESULTS(Bond_Context,Bond_C01_Trade,Bond_Requests,,Bond_Pricer)</f>
         <v/>
       </c>
       <c r="C22" s="7" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="34" customHeight="1">
       <c r="A23" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B22),",",", ")</f>
-        <v>=QS.EVALUATE("Bond.C01.Result", Bond_Pricer, Bond_C01_Trade, Bond_Context, Bond_Requests)</v>
+        <v>=QS.EVALUATE.RESULTS(Bond_Context, Bond_C01_Trade, Bond_Requests, , Bond_Pricer)</v>
       </c>
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
     </row>
     <row r="25" spans="1:3" ht="38" customHeight="1">
       <c r="A25" s="4" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B25" s="10" cm="1" t="str">
         <f t="array" ref="B25">_xll.QS.TRADE.CREATE("Bond.C02.Trade",Bond_Instrument,Bond_ValuationDate,Bond_Side,,,Bond_C02_Anchor,Bond_C02_AnchorValue)</f>
         <v/>
       </c>
       <c r="C25" s="7" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="34" customHeight="1">
@@ -2293,34 +2251,34 @@
     </row>
     <row r="28" spans="1:3" ht="38" customHeight="1">
       <c r="A28" s="4" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B28" s="10" cm="1" t="str">
-        <f t="array" ref="B28">_xll.QS.EVALUATE("Bond.C02.Result",Bond_Pricer,Bond_C02_Trade,Bond_Context,Bond_Requests)</f>
+        <f t="array" ref="B28">_xll.QS.EVALUATE.RESULTS(Bond_Context,Bond_C02_Trade,Bond_Requests,,Bond_Pricer)</f>
         <v/>
       </c>
       <c r="C28" s="7" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="34" customHeight="1">
       <c r="A29" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B28),",",", ")</f>
-        <v>=QS.EVALUATE("Bond.C02.Result", Bond_Pricer, Bond_C02_Trade, Bond_Context, Bond_Requests)</v>
+        <v>=QS.EVALUATE.RESULTS(Bond_Context, Bond_C02_Trade, Bond_Requests, , Bond_Pricer)</v>
       </c>
       <c r="B29" s="13"/>
       <c r="C29" s="13"/>
     </row>
     <row r="31" spans="1:3" ht="38" customHeight="1">
       <c r="A31" s="4" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B31" s="10" cm="1" t="str">
         <f t="array" ref="B31">_xll.QS.TRADE.CREATE("Bond.C03.Trade",Bond_Instrument,Bond_ValuationDate,Bond_Side,,,Bond_C03_Anchor,Bond_C03_AnchorValue)</f>
         <v/>
       </c>
       <c r="C31" s="7" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="34" customHeight="1">
@@ -2333,30 +2291,30 @@
     </row>
     <row r="34" spans="1:3" ht="38" customHeight="1">
       <c r="A34" s="4" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B34" s="10" cm="1" t="str">
-        <f t="array" ref="B34">_xll.QS.EVALUATE("Bond.C03.Result",Bond_Pricer,Bond_C03_Trade,Bond_Context,Bond_Requests)</f>
+        <f t="array" ref="B34">_xll.QS.EVALUATE.RESULTS(Bond_Context,Bond_C03_Trade,Bond_Requests,,Bond_Pricer)</f>
         <v/>
       </c>
       <c r="C34" s="7" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="34" customHeight="1">
       <c r="A35" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B34),",",", ")</f>
-        <v>=QS.EVALUATE("Bond.C03.Result", Bond_Pricer, Bond_C03_Trade, Bond_Context, Bond_Requests)</v>
+        <v>=QS.EVALUATE.RESULTS(Bond_Context, Bond_C03_Trade, Bond_Requests, , Bond_Pricer)</v>
       </c>
       <c r="B35" s="13"/>
       <c r="C35" s="13"/>
     </row>
     <row r="39" spans="1:3" ht="36" customHeight="1">
       <c r="A39" s="5" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C39" s="5"/>
     </row>
@@ -2389,14 +2347,14 @@
     </row>
     <row r="45" spans="1:3" ht="38" customHeight="1">
       <c r="A45" s="4" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B45" s="10">
         <f>INDEX(Bond_ResultHandles,MATCH(Bond_SelectedCase,Bond_CaseNames,0))</f>
         <v/>
       </c>
       <c r="C45" s="7" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="34" customHeight="1">
@@ -2453,7 +2411,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="38" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2463,7 +2421,7 @@
     </row>
     <row r="2" spans="1:6" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -2484,27 +2442,27 @@
         <v>36</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="36" customHeight="1">
       <c r="A6" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="D6" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="E6" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="F6" s="5" t="s">
         <v>125</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="34" customHeight="1">
@@ -2524,10 +2482,10 @@
         <v/>
       </c>
       <c r="E7" s="6" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="34" customHeight="1">
@@ -2547,10 +2505,10 @@
         <v/>
       </c>
       <c r="E8" s="6" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="34" customHeight="1">
@@ -2570,21 +2528,21 @@
         <v/>
       </c>
       <c r="E9" s="6" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="24" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B13" s="8" t="s">
         <v>59</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D13" s="7"/>
       <c r="E13" s="7"/>
@@ -2598,7 +2556,7 @@
     </row>
     <row r="17" spans="1:6" ht="24" customHeight="1">
       <c r="A17" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -2673,7 +2631,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="38" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2686,7 +2644,7 @@
     </row>
     <row r="2" spans="1:9" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -2713,19 +2671,19 @@
         <v>36</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="24" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B6" s="9">
         <f>Bond_SelectedCase</f>
         <v/>
       </c>
       <c r="C6" s="6" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="24" customHeight="1">
@@ -2768,14 +2726,14 @@
   <sheetData>
     <row r="1" spans="1:3" ht="38" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="2" spans="1:3" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -2792,14 +2750,14 @@
     </row>
     <row r="6" spans="1:3" ht="24" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B6" s="9">
         <f>Bond_SelectedCase</f>
         <v/>
       </c>
       <c r="C6" s="6" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="24" customHeight="1">

</xml_diff>

<commit_message>
fix(excel): repair examples and add Material ribbon icons
Correct zero-curve argument order in the generated pricing studies and validate
literal types against the registered worksheet signatures.

Keep pricing actions compact, reserve room for results at narrow pane sizes,
and select prepared markets and pricers from existing worksheet valuations.
Fix row selection updates and link worksheet errors to readable source cells.

Embed Google's Material Symbols Outlined in the ribbon, panel actions, tabs,
and copy menus, with local vector rendering and bundled Apache 2.0 notices.

Validated the Release build, panel/icon smoke tests at three pane sizes,
managed contracts, workbook and packaging tests, and a live Excel loan price.
</commit_message>
<xml_diff>
--- a/bindings/excel/examples/bond_pricing_example.xlsx
+++ b/bindings/excel/examples/bond_pricing_example.xlsx
@@ -1333,7 +1333,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F29"/>
-  <sheetFormatPr defaultRowHeight="26" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="26.25" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="8.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="22.7109375" style="1" customWidth="1"/>
@@ -1360,7 +1360,7 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
     </row>
-    <row r="3" spans="1:6" ht="26" customHeight="1">
+    <row r="3" spans="1:6" ht="26.25" customHeight="1">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -1370,7 +1370,7 @@
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="1:6" ht="26" customHeight="1">
+    <row r="4" spans="1:6" ht="26.25" customHeight="1">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -1378,7 +1378,7 @@
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
     </row>
-    <row r="6" spans="1:6" ht="26" customHeight="1">
+    <row r="6" spans="1:6" ht="26.25" customHeight="1">
       <c r="A6" s="4" t="s">
         <v>2</v>
       </c>
@@ -1388,7 +1388,7 @@
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" spans="1:6" ht="26" customHeight="1">
+    <row r="7" spans="1:6" ht="26.25" customHeight="1">
       <c r="A7" s="4"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -1396,7 +1396,7 @@
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
     </row>
-    <row r="9" spans="1:6" ht="26" customHeight="1">
+    <row r="9" spans="1:6" ht="26.25" customHeight="1">
       <c r="A9" s="5" t="s">
         <v>3</v>
       </c>
@@ -1406,7 +1406,7 @@
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
     </row>
-    <row r="10" spans="1:6" ht="34" customHeight="1">
+    <row r="10" spans="1:6" ht="33.75" customHeight="1">
       <c r="A10" s="4" t="s">
         <v>4</v>
       </c>
@@ -1420,7 +1420,7 @@
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
     </row>
-    <row r="11" spans="1:6" ht="34" customHeight="1">
+    <row r="11" spans="1:6" ht="33.75" customHeight="1">
       <c r="A11" s="4" t="s">
         <v>7</v>
       </c>
@@ -1434,7 +1434,7 @@
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
     </row>
-    <row r="12" spans="1:6" ht="34" customHeight="1">
+    <row r="12" spans="1:6" ht="33.75" customHeight="1">
       <c r="A12" s="4" t="s">
         <v>10</v>
       </c>
@@ -1448,7 +1448,7 @@
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
     </row>
-    <row r="13" spans="1:6" ht="34" customHeight="1">
+    <row r="13" spans="1:6" ht="33.75" customHeight="1">
       <c r="A13" s="4" t="s">
         <v>13</v>
       </c>
@@ -1462,7 +1462,7 @@
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
     </row>
-    <row r="14" spans="1:6" ht="34" customHeight="1">
+    <row r="14" spans="1:6" ht="33.75" customHeight="1">
       <c r="A14" s="4" t="s">
         <v>16</v>
       </c>
@@ -1476,7 +1476,7 @@
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
     </row>
-    <row r="15" spans="1:6" ht="34" customHeight="1">
+    <row r="15" spans="1:6" ht="33.75" customHeight="1">
       <c r="A15" s="4" t="s">
         <v>19</v>
       </c>
@@ -1490,7 +1490,7 @@
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
     </row>
-    <row r="18" spans="1:6" ht="26" customHeight="1">
+    <row r="18" spans="1:6" ht="26.25" customHeight="1">
       <c r="A18" s="5" t="s">
         <v>22</v>
       </c>
@@ -1536,7 +1536,7 @@
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
     </row>
-    <row r="23" spans="1:6" ht="26" customHeight="1">
+    <row r="23" spans="1:6" ht="26.25" customHeight="1">
       <c r="A23" s="5" t="s">
         <v>29</v>
       </c>
@@ -1546,7 +1546,7 @@
       <c r="E23" s="5"/>
       <c r="F23" s="5"/>
     </row>
-    <row r="24" spans="1:6" ht="34" customHeight="1">
+    <row r="24" spans="1:6" ht="33.75" customHeight="1">
       <c r="A24" s="1" t="s">
         <v>30</v>
       </c>
@@ -1556,7 +1556,7 @@
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
     </row>
-    <row r="25" spans="1:6" ht="34" customHeight="1">
+    <row r="25" spans="1:6" ht="33.75" customHeight="1">
       <c r="A25" s="1" t="s">
         <v>31</v>
       </c>
@@ -1566,7 +1566,7 @@
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
     </row>
-    <row r="26" spans="1:6" ht="34" customHeight="1">
+    <row r="26" spans="1:6" ht="33.75" customHeight="1">
       <c r="A26" s="1" t="s">
         <v>32</v>
       </c>
@@ -1576,7 +1576,7 @@
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
     </row>
-    <row r="28" spans="1:6" ht="26" customHeight="1">
+    <row r="28" spans="1:6" ht="26.25" customHeight="1">
       <c r="A28" s="7" t="s">
         <v>33</v>
       </c>
@@ -1586,7 +1586,7 @@
       <c r="E28" s="7"/>
       <c r="F28" s="7"/>
     </row>
-    <row r="29" spans="1:6" ht="26" customHeight="1">
+    <row r="29" spans="1:6" ht="26.25" customHeight="1">
       <c r="A29" s="7"/>
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
@@ -1652,7 +1652,7 @@
     <col min="3" max="3" width="62.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="38" customHeight="1">
+    <row r="1" spans="1:3" ht="38.25" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>34</v>
       </c>
@@ -1690,7 +1690,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="32" customHeight="1">
+    <row r="7" spans="1:3" ht="32.25" customHeight="1">
       <c r="A7" s="1" t="s">
         <v>41</v>
       </c>
@@ -1701,7 +1701,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="32" customHeight="1">
+    <row r="8" spans="1:3" ht="32.25" customHeight="1">
       <c r="A8" s="1" t="s">
         <v>44</v>
       </c>
@@ -1712,7 +1712,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="32" customHeight="1">
+    <row r="9" spans="1:3" ht="32.25" customHeight="1">
       <c r="A9" s="1" t="s">
         <v>46</v>
       </c>
@@ -1723,7 +1723,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="32" customHeight="1">
+    <row r="10" spans="1:3" ht="32.25" customHeight="1">
       <c r="A10" s="1" t="s">
         <v>49</v>
       </c>
@@ -1734,7 +1734,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="32" customHeight="1">
+    <row r="11" spans="1:3" ht="32.25" customHeight="1">
       <c r="A11" s="1" t="s">
         <v>51</v>
       </c>
@@ -1745,7 +1745,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="32" customHeight="1">
+    <row r="12" spans="1:3" ht="32.25" customHeight="1">
       <c r="A12" s="1" t="s">
         <v>53</v>
       </c>
@@ -1898,7 +1898,7 @@
     <col min="3" max="3" width="44.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="38" customHeight="1">
+    <row r="1" spans="1:3" ht="38.25" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>78</v>
       </c>
@@ -1997,7 +1997,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="38" customHeight="1">
+    <row r="18" spans="1:3" ht="38.25" customHeight="1">
       <c r="A18" s="4" t="s">
         <v>92</v>
       </c>
@@ -2009,7 +2009,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="34" customHeight="1">
+    <row r="19" spans="1:3" ht="33.75" customHeight="1">
       <c r="A19" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B18),",",", ")</f>
         <v>=QS.CONTEXT.CREATE("Bond.Root", Bond_ValuationDate, "USD", "SOFR")</v>
@@ -2017,22 +2017,22 @@
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
     </row>
-    <row r="21" spans="1:3" ht="38" customHeight="1">
+    <row r="21" spans="1:3" ht="38.25" customHeight="1">
       <c r="A21" s="4" t="s">
         <v>94</v>
       </c>
       <c r="B21" s="10" cm="1" t="str">
-        <f t="array" ref="B21">_xll.QS.CONTEXT.ADD.ZERO.CURVE(Bond_Root,"SOFR",Bond_Pillars,Bond_ZeroRates,"Actual360","Linear",TRUE,"Continuous","Annual")</f>
+        <f t="array" ref="B21">_xll.QS.CONTEXT.ADD.ZERO.CURVE(Bond_Root,"SOFR",Bond_Pillars,Bond_ZeroRates,"Actual360","Continuous","Annual","Linear",TRUE)</f>
         <v/>
       </c>
       <c r="C21" s="7" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="34" customHeight="1">
+    <row r="22" spans="1:3" ht="33.75" customHeight="1">
       <c r="A22" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B21),",",", ")</f>
-        <v>=QS.CONTEXT.ADD.ZERO.CURVE(Bond_Root, "SOFR", Bond_Pillars, Bond_ZeroRates, "Actual360", "Linear", TRUE, "Continuous", "Annual")</v>
+        <v>=QS.CONTEXT.ADD.ZERO.CURVE(Bond_Root, "SOFR", Bond_Pillars, Bond_ZeroRates, "Actual360", "Continuous", "Annual", "Linear", TRUE)</v>
       </c>
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
@@ -2071,7 +2071,7 @@
     <col min="2" max="3" width="48.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="38" customHeight="1">
+    <row r="1" spans="1:3" ht="38.25" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>96</v>
       </c>
@@ -2109,7 +2109,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="38" customHeight="1">
+    <row r="7" spans="1:3" ht="38.25" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>101</v>
       </c>
@@ -2121,7 +2121,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="34" customHeight="1">
+    <row r="8" spans="1:3" ht="33.75" customHeight="1">
       <c r="A8" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B7),",",", ")</f>
         <v>=QS.CONTEXT.PREPARE("Bond.Context", Bond_Root, Bond_MarketInputs)</v>
@@ -2129,7 +2129,7 @@
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
     </row>
-    <row r="10" spans="1:3" ht="38" customHeight="1">
+    <row r="10" spans="1:3" ht="38.25" customHeight="1">
       <c r="A10" s="4" t="s">
         <v>103</v>
       </c>
@@ -2141,7 +2141,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="34" customHeight="1">
+    <row r="11" spans="1:3" ht="33.75" customHeight="1">
       <c r="A11" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B10),",",", ")</f>
         <v>=QS.INSTRUMENT.FIXED.RATE.BOND("Bond.Instrument", Bond_Start, Bond_Maturity, "USD", , Bond_Notional, Bond_Coupon, "Actual360", "Compounded", "Semiannual", "Semiannual")</v>
@@ -2149,7 +2149,7 @@
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
     </row>
-    <row r="13" spans="1:3" ht="38" customHeight="1">
+    <row r="13" spans="1:3" ht="38.25" customHeight="1">
       <c r="A13" s="4" t="s">
         <v>105</v>
       </c>
@@ -2161,7 +2161,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="34" customHeight="1">
+    <row r="14" spans="1:3" ht="33.75" customHeight="1">
       <c r="A14" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B13),",",", ")</f>
         <v>=QS.DISCOUNT.POLICY.FIXED.INCOME("Bond.Policy", Bond_DiscountCurrency, Bond_DiscountIndex)</v>
@@ -2169,7 +2169,7 @@
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>
     </row>
-    <row r="16" spans="1:3" ht="38" customHeight="1">
+    <row r="16" spans="1:3" ht="38.25" customHeight="1">
       <c r="A16" s="4" t="s">
         <v>107</v>
       </c>
@@ -2181,7 +2181,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="34" customHeight="1">
+    <row r="17" spans="1:3" ht="33.75" customHeight="1">
       <c r="A17" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B16),",",", ")</f>
         <v>=QS.PRICER.CREATE("Bond.Pricer", "BondPricer", Bond_Policy)</v>
@@ -2189,7 +2189,7 @@
       <c r="B17" s="13"/>
       <c r="C17" s="13"/>
     </row>
-    <row r="19" spans="1:3" ht="38" customHeight="1">
+    <row r="19" spans="1:3" ht="38.25" customHeight="1">
       <c r="A19" s="4" t="s">
         <v>109</v>
       </c>
@@ -2201,7 +2201,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="34" customHeight="1">
+    <row r="20" spans="1:3" ht="33.75" customHeight="1">
       <c r="A20" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B19),",",", ")</f>
         <v>=QS.TRADE.CREATE("Bond.C01.Trade", Bond_Instrument, Bond_ValuationDate, Bond_Side, , , Bond_C01_Anchor, Bond_C01_AnchorValue)</v>
@@ -2209,7 +2209,7 @@
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
     </row>
-    <row r="22" spans="1:3" ht="38" customHeight="1">
+    <row r="22" spans="1:3" ht="38.25" customHeight="1">
       <c r="A22" s="4" t="s">
         <v>111</v>
       </c>
@@ -2221,7 +2221,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="34" customHeight="1">
+    <row r="23" spans="1:3" ht="33.75" customHeight="1">
       <c r="A23" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B22),",",", ")</f>
         <v>=QS.EVALUATE.RESULTS(Bond_Context, Bond_C01_Trade, Bond_Requests, , Bond_Pricer)</v>
@@ -2229,7 +2229,7 @@
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
     </row>
-    <row r="25" spans="1:3" ht="38" customHeight="1">
+    <row r="25" spans="1:3" ht="38.25" customHeight="1">
       <c r="A25" s="4" t="s">
         <v>113</v>
       </c>
@@ -2241,7 +2241,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="34" customHeight="1">
+    <row r="26" spans="1:3" ht="33.75" customHeight="1">
       <c r="A26" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B25),",",", ")</f>
         <v>=QS.TRADE.CREATE("Bond.C02.Trade", Bond_Instrument, Bond_ValuationDate, Bond_Side, , , Bond_C02_Anchor, Bond_C02_AnchorValue)</v>
@@ -2249,7 +2249,7 @@
       <c r="B26" s="13"/>
       <c r="C26" s="13"/>
     </row>
-    <row r="28" spans="1:3" ht="38" customHeight="1">
+    <row r="28" spans="1:3" ht="38.25" customHeight="1">
       <c r="A28" s="4" t="s">
         <v>114</v>
       </c>
@@ -2261,7 +2261,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="34" customHeight="1">
+    <row r="29" spans="1:3" ht="33.75" customHeight="1">
       <c r="A29" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B28),",",", ")</f>
         <v>=QS.EVALUATE.RESULTS(Bond_Context, Bond_C02_Trade, Bond_Requests, , Bond_Pricer)</v>
@@ -2269,7 +2269,7 @@
       <c r="B29" s="13"/>
       <c r="C29" s="13"/>
     </row>
-    <row r="31" spans="1:3" ht="38" customHeight="1">
+    <row r="31" spans="1:3" ht="38.25" customHeight="1">
       <c r="A31" s="4" t="s">
         <v>115</v>
       </c>
@@ -2281,7 +2281,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="34" customHeight="1">
+    <row r="32" spans="1:3" ht="33.75" customHeight="1">
       <c r="A32" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B31),",",", ")</f>
         <v>=QS.TRADE.CREATE("Bond.C03.Trade", Bond_Instrument, Bond_ValuationDate, Bond_Side, , , Bond_C03_Anchor, Bond_C03_AnchorValue)</v>
@@ -2289,7 +2289,7 @@
       <c r="B32" s="13"/>
       <c r="C32" s="13"/>
     </row>
-    <row r="34" spans="1:3" ht="38" customHeight="1">
+    <row r="34" spans="1:3" ht="38.25" customHeight="1">
       <c r="A34" s="4" t="s">
         <v>116</v>
       </c>
@@ -2301,7 +2301,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="34" customHeight="1">
+    <row r="35" spans="1:3" ht="33.75" customHeight="1">
       <c r="A35" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B34),",",", ")</f>
         <v>=QS.EVALUATE.RESULTS(Bond_Context, Bond_C03_Trade, Bond_Requests, , Bond_Pricer)</v>
@@ -2345,7 +2345,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="38" customHeight="1">
+    <row r="45" spans="1:3" ht="38.25" customHeight="1">
       <c r="A45" s="4" t="s">
         <v>132</v>
       </c>
@@ -2357,7 +2357,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="34" customHeight="1">
+    <row r="46" spans="1:3" ht="33.75" customHeight="1">
       <c r="A46" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B45),",",", ")</f>
         <v>=INDEX(Bond_ResultHandles, MATCH(Bond_SelectedCase, Bond_CaseNames, 0))</v>
@@ -2409,7 +2409,7 @@
     <col min="5" max="6" width="16.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="38" customHeight="1">
+    <row r="1" spans="1:6" ht="38.25" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>117</v>
       </c>
@@ -2465,7 +2465,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="34" customHeight="1">
+    <row r="7" spans="1:6" ht="33.75" customHeight="1">
       <c r="A7" s="1" t="s">
         <v>59</v>
       </c>
@@ -2488,7 +2488,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="34" customHeight="1">
+    <row r="8" spans="1:6" ht="33.75" customHeight="1">
       <c r="A8" s="1" t="s">
         <v>61</v>
       </c>
@@ -2511,7 +2511,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="34" customHeight="1">
+    <row r="9" spans="1:6" ht="33.75" customHeight="1">
       <c r="A9" s="1" t="s">
         <v>62</v>
       </c>
@@ -2629,7 +2629,7 @@
     <col min="9" max="9" width="8.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="38" customHeight="1">
+    <row r="1" spans="1:9" ht="38.25" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>135</v>
       </c>
@@ -2724,7 +2724,7 @@
     <col min="3" max="3" width="24.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="38" customHeight="1">
+    <row r="1" spans="1:3" ht="38.25" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>140</v>
       </c>

</xml_diff>